<commit_message>
chore: atualiza planilha de fretes por cidade Hidracor
</commit_message>
<xml_diff>
--- a/public/Fretes por Cidade Hidracor.xlsx
+++ b/public/Fretes por Cidade Hidracor.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\DEV\MIDAS RENT A CAR\midas-log\public\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{732A7D15-5868-43C0-BC3E-96967AA5A0E1}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7E7B5C06-E651-4BAA-9723-324D3CC7BA12}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" tabRatio="795" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1681,22 +1681,22 @@
         <v>60</v>
       </c>
       <c r="C15" s="7">
-        <v>232.60474006000001</v>
+        <v>233</v>
       </c>
       <c r="D15" s="7">
-        <v>244.84709480000001</v>
+        <v>245</v>
       </c>
       <c r="E15" s="7">
-        <v>257.73378400000001</v>
+        <v>258</v>
       </c>
       <c r="F15" s="7">
-        <v>271.29872</v>
+        <v>271</v>
       </c>
       <c r="G15" s="7">
-        <v>285.57760000000002</v>
+        <v>286</v>
       </c>
       <c r="H15" s="7">
-        <v>300.608</v>
+        <v>301</v>
       </c>
     </row>
     <row r="16" spans="1:8" x14ac:dyDescent="0.25">
@@ -1915,22 +1915,22 @@
         <v>61</v>
       </c>
       <c r="C24" s="7">
-        <v>259.29708728000003</v>
+        <v>259</v>
       </c>
       <c r="D24" s="7">
-        <v>272.94430240000003</v>
+        <v>273</v>
       </c>
       <c r="E24" s="7">
-        <v>287.30979200000002</v>
+        <v>287</v>
       </c>
       <c r="F24" s="7">
-        <v>302.43136000000004</v>
+        <v>302</v>
       </c>
       <c r="G24" s="7">
-        <v>318.34880000000004</v>
+        <v>318</v>
       </c>
       <c r="H24" s="7">
-        <v>335.10400000000004</v>
+        <v>335</v>
       </c>
     </row>
     <row r="25" spans="1:8" x14ac:dyDescent="0.25">
@@ -2461,22 +2461,22 @@
         <v>62</v>
       </c>
       <c r="C45" s="7">
-        <v>240.23112498000003</v>
+        <v>240</v>
       </c>
       <c r="D45" s="7">
-        <v>252.87486840000003</v>
+        <v>253</v>
       </c>
       <c r="E45" s="7">
-        <v>266.18407200000001</v>
+        <v>266</v>
       </c>
       <c r="F45" s="7">
-        <v>280.19376</v>
+        <v>280</v>
       </c>
       <c r="G45" s="7">
-        <v>294.94080000000002</v>
+        <v>295</v>
       </c>
       <c r="H45" s="7">
-        <v>310.464</v>
+        <v>310</v>
       </c>
     </row>
     <row r="46" spans="1:8" s="4" customFormat="1" x14ac:dyDescent="0.25">

</xml_diff>